<commit_message>
Claude: figuras y código de figuras (3.B.3)
</commit_message>
<xml_diff>
--- a/Ejercicio-3/Parte-B/3.B.3/Code/datos_3B3.xlsx
+++ b/Ejercicio-3/Parte-B/3.B.3/Code/datos_3B3.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Léeme'!$A$1:$B$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fuentes'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Series_brutas'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cifras_citadas'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cifras_citadas'!$A$1:$F$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -870,15 +870,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="67" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1273,8 +1273,342 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Valor del ahorro fiscal de la deuda</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>% del valor de la empresa</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>GRAHAM (2000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Valor del ahorro fiscal de la deuda, neto de impuestos personales</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>% del valor de la empresa</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>GRAHAM (2000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>VA de las dificultades financieras, empresa BBB, ajustado por riesgo</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>% del valor previo a las dificultades</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ALMEIDA y PHILIPPON (2007)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>VA de las dificultades financieras, empresa BBB, sin primas de riesgo</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>% del valor previo a las dificultades</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ALMEIDA y PHILIPPON (2007)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Costes directos de quiebra, ferrocarriles de EE. UU. (mínimo y máximo)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1-5,3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>% del valor de la empresa</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>WARNER (1977)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Costes de las dificultades financieras, estimación preferida</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>% del valor de la empresa</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ANDRADE y KAPLAN (1998), versión de documento de trabajo del NBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Límite a la deducción de gastos financieros netos</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>% del beneficio operativo</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Art. 16 Ley 27/2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Gastos financieros netos deducibles en todo caso</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>millón de euros</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Art. 16 Ley 27/2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Reserva de capitalización, reducción general</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>% del aumento de fondos propios</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Art. 25 Ley 27/2014 (desde 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bloque 2, «Impuestos e insolvencia»</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Reserva de capitalización, reducción máxima con aumento de plantilla</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>% del aumento de fondos propios</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Art. 25 Ley 27/2014 (desde 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bloque 2, «MODIGLIANI y MILLER (1958)», nota</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Empresas con calificación AAA de S&amp;P, hace cuatro décadas y en 2020</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>65 y 5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>empresas</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>WIGGLESWORTH (2020), Financial Times</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F13"/>
+  <autoFilter ref="A1:F24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>